<commit_message>
feat: change to coverage version
</commit_message>
<xml_diff>
--- a/src/rag_results.xlsx
+++ b/src/rag_results.xlsx
@@ -1,47 +1,107 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yiting/Desktop/rag 2/src/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFC9C7FD-2FCA-C44C-A12C-D32C5039023F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="4300" yWindow="880" windowWidth="29900" windowHeight="20240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Results" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+  <si>
+    <t>商品代號</t>
+  </si>
+  <si>
+    <t>問題（original)</t>
+  </si>
+  <si>
+    <t>回答(final)</t>
+  </si>
+  <si>
+    <t>檢索條款(final)</t>
+  </si>
+  <si>
+    <t>是否 reAct</t>
+  </si>
+  <si>
+    <t>initial answer</t>
+  </si>
+  <si>
+    <t>reviseAnswer1</t>
+  </si>
+  <si>
+    <t>reviseAnswer2</t>
+  </si>
+  <si>
+    <t>評估結果(final)</t>
+  </si>
+  <si>
+    <t>coverage_score(final)</t>
+  </si>
+  <si>
+    <t>C_fact(final)</t>
+  </si>
+  <si>
+    <t>C_conf(final)</t>
+  </si>
+  <si>
+    <t>timestamp</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="176" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
-      <name val="Calibri"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="新細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -54,98 +114,43 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -433,164 +438,77 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="8" width="40" customWidth="1"/>
+    <col min="9" max="9" width="24" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="12" width="16" customWidth="1"/>
+    <col min="13" max="13" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>商品代號</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>問題（original)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>回答(final)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>檢索條款(final)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>是否 reAct</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>initial answer</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>reviseAnswer1</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>reviseAnswer2</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>評估結果(final)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>coverage_score(final)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>C_fact(final)</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>C_conf(final)</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SC1</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>保戶在114/1/10投保樂鍾溢，如果他在115/3/30罹患特定傷病的話，他在115/1/9會領到無理賠回饋保險金嗎?</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>回答：  
-1. 樂鍾溢保單包含「無理賠回饋保險金」的條款，依據第十四條規定，若被保險人在保險單年度末仍生存且未曾申領「特定傷病保險金」，可獲得「無理賠回饋保險金」。  
-2. 115/1/9屬於保險單年度末，需確認被保險人在該日期前是否符合條件。由於被保險人在115/3/30罹患特定傷病，且診斷日期晚於115/1/9，因此115/1/9時未曾申領「特定傷病保險金」，符合給付條件。  
-3. 115/3/30罹患特定傷病不影響115/1/9的「無理賠回饋保險金」給付資格，但若事後發現被保險人不符條件，保險公司有權要求返還或扣回該保險金。  
-4. 保單生效日期為114/1/10，等待期為30日，故114/2/9起保單進入有效期間，與本問題無直接影響。  
-條文依據：  
-- [第十四條 無理賠回饋保險金的給付]  
-- [第十二條 特定傷病保險金的給付]</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>第十四條 無理賠回饋保險金的給付 | payout_items | 第二十條 無理賠回饋保險金的申領 | 第十二條 特定傷病保險金的給付 | other_metadata</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>回答：  
-1. 樂鍾溢保單包含「無理賠回饋保險金」的條款，依據第十四條規定，若被保險人在保險單年度末仍生存且未曾申領「特定傷病保險金」，可獲得「無理賠回饋保險金」。  
-2. 115/1/9屬於保險單年度末，需確認被保險人在該日期前是否符合條件。由於被保險人在115/3/30罹患特定傷病，且診斷日期晚於115/1/9，因此115/1/9時未曾申領「特定傷病保險金」，符合給付條件。  
-3. 115/3/30罹患特定傷病不影響115/1/9的「無理賠回饋保險金」給付資格，但若事後發現被保險人不符條件，保險公司有權要求返還或扣回該保險金。  
-4. 保單生效日期為114/1/10，等待期為30日，故114/2/9起保單進入有效期間，與本問題無直接影響。  
-條文依據：  
-- [第十四條 無理賠回饋保險金的給付]  
-- [第十二條 特定傷病保險金的給付]</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>{"points": [{"id": "1", "point": "確認樂鍾溢保單是否包含無理賠回饋保險金的條款", "must_have": true, "分數": 1.0}, {"id": "2", "point": "確認115/1/9是否符合無理賠回饋保險金的給付條件", "must_have": true, "分數": 1.0}, {"id": "3", "point": "確認115/3/30罹患特定傷病是否影響無理賠回饋保險金的給付資格", "must_have": true, "分數": 1.0}, {"id": "4", "point": "確認保單的生效日期及相關等待期規定", "must_have": false, "分數": 1.0}], "coverage_score": 1.0, "nli": {"entailment": 0.930912, "neutral": 0.061623, "contradiction": 0.007465, "factuality": 0.992535, "C_fact": 0.992535}, "C_conf": 0.9955}</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" s="3" t="n">
-        <v>0.9925349999999999</v>
-      </c>
-      <c r="L2" s="3" t="n">
-        <v>0.9955000000000001</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>2026-03-15 11:33:12</t>
-        </is>
-      </c>
+    <row r="2" spans="1:13">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: change to factual version
</commit_message>
<xml_diff>
--- a/src/rag_results.xlsx
+++ b/src/rag_results.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -590,6 +590,65 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AGG</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>保障範圍包括哪些？</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>回答：  
+保障範圍包括：住院醫療保險金、加護病房或燒燙傷病房保險金、祝壽保險金、身故保險金或喪葬費用保險金，以及所繳保險費的退還。
+條文依據：  
+- [第五條 保險範圍]  
+- [摘要]</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>payout_items | 第五條 保險範圍 | 第二條 名詞定義 | summary | 第十八條 除外責任（一）</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>回答：  
+保障範圍包括：住院醫療保險金、加護病房或燒燙傷病房保險金、祝壽保險金、身故保險金或喪葬費用保險金，以及所繳保險費的退還。
+條文依據：  
+- [第五條 保險範圍]  
+- [摘要]</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>{"nli": {"entailment": 0.299185, "neutral": 0.699514, "contradiction": 0.0013, "factuality": 0.9987, "C_fact": 0.9987}, "C_conf": 0.9987}</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n">
+        <v>0.9987</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>0.9987</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-03-21 17:26:45</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>